<commit_message>
excel file update,add jacoco
</commit_message>
<xml_diff>
--- a/src/test/resources/inputdata1.xlsx
+++ b/src/test/resources/inputdata1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\桌面\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\COMP\AI-based-Scheduling-System\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDE58C07-55B9-410B-B6A2-6127D2D12D44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F538A81D-7C2E-46DC-A2EB-DEFE6683CBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1120" yWindow="420" windowWidth="23560" windowHeight="14680" activeTab="2" xr2:uid="{04D44C14-949C-4A62-82BE-A38901EFB31F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{04D44C14-949C-4A62-82BE-A38901EFB31F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -196,11 +196,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -209,20 +209,20 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -281,9 +281,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主题">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -321,7 +321,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -427,7 +427,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -569,7 +569,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -578,24 +578,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1B12756-D463-42B3-8131-D595FCB9EDB5}">
   <dimension ref="A1:N7"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" customWidth="1"/>
-    <col min="3" max="3" width="14.5" customWidth="1"/>
-    <col min="4" max="4" width="14.58203125" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" customWidth="1"/>
-    <col min="6" max="6" width="10.75" customWidth="1"/>
-    <col min="7" max="7" width="11.1640625" customWidth="1"/>
-    <col min="9" max="9" width="13.08203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="11.33203125" customWidth="1"/>
-    <col min="12" max="12" width="11.5" customWidth="1"/>
-    <col min="13" max="13" width="10.33203125" customWidth="1"/>
-    <col min="14" max="14" width="16.25" customWidth="1"/>
+    <col min="1" max="1" width="22.6328125" customWidth="1"/>
+    <col min="2" max="2" width="16.36328125" customWidth="1"/>
+    <col min="3" max="3" width="14.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" customWidth="1"/>
+    <col min="5" max="5" width="12.36328125" customWidth="1"/>
+    <col min="6" max="6" width="10.7265625" customWidth="1"/>
+    <col min="7" max="7" width="11.1796875" customWidth="1"/>
+    <col min="9" max="9" width="13.08984375" customWidth="1"/>
+    <col min="10" max="10" width="16.81640625" customWidth="1"/>
+    <col min="11" max="11" width="11.36328125" customWidth="1"/>
+    <col min="12" max="12" width="11.453125" customWidth="1"/>
+    <col min="13" max="13" width="10.36328125" customWidth="1"/>
+    <col min="14" max="14" width="16.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -639,7 +639,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -680,7 +680,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -718,7 +718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -756,7 +756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -794,7 +794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -832,7 +832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -879,14 +879,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B67BDCC-FEB8-4CC2-A8A1-822369E85BAD}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="15.08203125" customWidth="1"/>
+    <col min="1" max="1" width="15.08984375" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="13.5" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>36</v>
       </c>
@@ -897,7 +897,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2">
         <v>10</v>
       </c>
@@ -908,100 +908,100 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3">
         <v>30</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4">
         <v>18</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5">
         <v>25</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
       <c r="A6">
         <v>20</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C6" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="A7">
         <v>22</v>
       </c>
       <c r="B7">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3">
       <c r="A8">
         <v>16</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3">
       <c r="A9">
         <v>18</v>
       </c>
       <c r="B9">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="C9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3">
       <c r="A10">
         <v>24</v>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C10" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3">
       <c r="A11">
         <v>25</v>
       </c>
       <c r="B11">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C11" t="s">
         <v>43</v>
@@ -1016,140 +1016,140 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0398738-4E45-4A9D-9CE5-9928B7D8976A}">
   <dimension ref="A1:B24"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="21.6640625" customWidth="1"/>
+    <col min="1" max="1" width="21.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" s="3">
         <v>45329</v>
       </c>
       <c r="B2" s="2"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2">
       <c r="A3" s="3">
         <v>45330</v>
       </c>
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2">
       <c r="A4" s="3">
         <v>45331</v>
       </c>
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2">
       <c r="A5" s="3">
         <v>45332</v>
       </c>
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2">
       <c r="A6" s="3">
         <v>45333</v>
       </c>
       <c r="B6" s="2"/>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2">
       <c r="A7" s="3">
         <v>45334</v>
       </c>
       <c r="B7" s="2"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2">
       <c r="A8" s="3">
         <v>45335</v>
       </c>
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2">
       <c r="A9" s="3">
         <v>45336</v>
       </c>
       <c r="B9" s="2"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2">
       <c r="A10" s="3">
         <v>45337</v>
       </c>
       <c r="B10" s="2"/>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2">
       <c r="A11" s="3">
         <v>45338</v>
       </c>
       <c r="B11" s="2"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2">
       <c r="A12" s="3">
         <v>45339</v>
       </c>
       <c r="B12" s="2"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2">
       <c r="A13" s="3">
         <v>45340</v>
       </c>
       <c r="B13" s="2"/>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2">
       <c r="A14" s="3">
         <v>45341</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2">
       <c r="A15" s="3">
         <v>45342</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2">
       <c r="A16" s="3">
         <v>45343</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1">
       <c r="A17" s="3">
         <v>45344</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1">
       <c r="A18" s="3">
         <v>45345</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1">
       <c r="A19" s="3">
         <v>45346</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1">
       <c r="A20" s="3">
         <v>45347</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1">
       <c r="A21" s="3">
         <v>45348</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1">
       <c r="A22" s="3">
         <v>45349</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1">
       <c r="A23" s="3">
         <v>45350</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1">
       <c r="A24" s="3">
         <v>45351</v>
       </c>

</xml_diff>